<commit_message>
Change currency from USD to ZAR across all sheets
Co-authored-by: iiwiiInsider <163913868+iiwiiInsider@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Weekly_Intraday_Trading_Journal.xlsx
+++ b/Weekly_Intraday_Trading_Journal.xlsx
@@ -20,8 +20,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="R #,##0.00"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -95,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -113,6 +114,7 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -587,7 +589,7 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>P&amp;L ($)</t>
+          <t>P&amp;L (R)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -645,7 +647,6 @@
       <c r="A2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2">
         <f>IF(B2="","",TEXT(B2,"dddd"))</f>
         <v/>
@@ -3197,7 +3198,6 @@
           <t>Week Starting:</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -3223,10 +3223,9 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Daily Profit Target ($):</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>Daily Profit Target (R):</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -3240,10 +3239,9 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Daily Loss Limit ($):</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>Daily Loss Limit (R):</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -3260,7 +3258,6 @@
           <t>Max Trades Per Day:</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -3277,20 +3274,18 @@
           <t>Focus Setup:</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr"/>
       <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Total P&amp;L ($):</t>
-        </is>
-      </c>
-      <c r="B11" s="5">
+          <t>Total P&amp;L (R):</t>
+        </is>
+      </c>
+      <c r="B11" s="11">
         <f>SUM('Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3299,28 +3294,26 @@
           <t>What Went Well:</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Total Fees ($):</t>
-        </is>
-      </c>
-      <c r="B12" s="5">
+          <t>Total Fees (R):</t>
+        </is>
+      </c>
+      <c r="B12" s="11">
         <f>SUM('Trade Log'!P:P)</f>
         <v/>
       </c>
       <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Net P&amp;L ($):</t>
-        </is>
-      </c>
-      <c r="B13" s="5">
+          <t>Net P&amp;L (R):</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
         <f>B11-B12</f>
         <v/>
       </c>
@@ -3329,20 +3322,18 @@
           <t>What Needs Improvement:</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr"/>
       <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Average Win ($):</t>
-        </is>
-      </c>
-      <c r="B15" s="5">
+          <t>Average Win (R):</t>
+        </is>
+      </c>
+      <c r="B15" s="11">
         <f>AVERAGEIF('Trade Log'!M:M,"&gt;0",'Trade Log'!M:M)</f>
         <v/>
       </c>
@@ -3351,15 +3342,14 @@
           <t>Key Lessons:</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Average Loss ($):</t>
-        </is>
-      </c>
-      <c r="B16" s="5">
+          <t>Average Loss (R):</t>
+        </is>
+      </c>
+      <c r="B16" s="11">
         <f>AVERAGEIF('Trade Log'!M:M,"&lt;0",'Trade Log'!M:M)</f>
         <v/>
       </c>
@@ -3370,7 +3360,7 @@
           <t>Avg R:R Ratio:</t>
         </is>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="11">
         <f>AVERAGE('Trade Log'!O:O)</f>
         <v/>
       </c>
@@ -3381,7 +3371,7 @@
           <t>Profit Factor:</t>
         </is>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="11">
         <f>IF(ABS(B16)=0,0,B15/ABS(B16))</f>
         <v/>
       </c>
@@ -3392,10 +3382,10 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Largest Win ($):</t>
-        </is>
-      </c>
-      <c r="B20" s="5">
+          <t>Largest Win (R):</t>
+        </is>
+      </c>
+      <c r="B20" s="11">
         <f>MAX('Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3403,10 +3393,10 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Largest Loss ($):</t>
-        </is>
-      </c>
-      <c r="B21" s="5">
+          <t>Largest Loss (R):</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
         <f>MIN('Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3456,7 +3446,6 @@
           <t>Month/Year:</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3476,12 +3465,12 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Net P&amp;L ($)</t>
+          <t>Net P&amp;L (R)</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Cumulative P&amp;L ($)</t>
+          <t>Cumulative P&amp;L (R)</t>
         </is>
       </c>
     </row>
@@ -3491,10 +3480,8 @@
           <t>Week 1</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" s="5" t="inlineStr"/>
-      <c r="E6" s="5">
+      <c r="D6" s="11" t="inlineStr"/>
+      <c r="E6" s="11">
         <f>SUM($D$6:D6)</f>
         <v/>
       </c>
@@ -3505,10 +3492,8 @@
           <t>Week 2</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" s="5" t="inlineStr"/>
-      <c r="E7" s="5">
+      <c r="D7" s="11" t="inlineStr"/>
+      <c r="E7" s="11">
         <f>SUM($D$6:D7)</f>
         <v/>
       </c>
@@ -3519,10 +3504,8 @@
           <t>Week 3</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" s="5" t="inlineStr"/>
-      <c r="E8" s="5">
+      <c r="D8" s="11" t="inlineStr"/>
+      <c r="E8" s="11">
         <f>SUM($D$6:D8)</f>
         <v/>
       </c>
@@ -3533,10 +3516,8 @@
           <t>Week 4</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" s="5" t="inlineStr"/>
-      <c r="E9" s="5">
+      <c r="D9" s="11" t="inlineStr"/>
+      <c r="E9" s="11">
         <f>SUM($D$6:D9)</f>
         <v/>
       </c>
@@ -3547,10 +3528,8 @@
           <t>Week 5</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5">
+      <c r="D10" s="11" t="inlineStr"/>
+      <c r="E10" s="11">
         <f>SUM($D$6:D10)</f>
         <v/>
       </c>
@@ -3565,11 +3544,11 @@
         <f>SUM(B6:B10)</f>
         <v/>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="11">
         <f>SUM(D6:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="11">
         <f>E10</f>
         <v/>
       </c>
@@ -3638,7 +3617,7 @@
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Total P&amp;L ($)</t>
+          <t>Total P&amp;L (R)</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
@@ -3658,7 +3637,7 @@
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Net P&amp;L ($)</t>
+          <t>Net P&amp;L (R)</t>
         </is>
       </c>
     </row>
@@ -3676,7 +3655,7 @@
         <f>IF(B6=0,0,COUNTIFS('Trade Log'!R:R,A6,'Trade Log'!M:M,"&gt;0")/B6*100)</f>
         <v/>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="11">
         <f>SUMIF('Trade Log'!R:R,A6,'Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3695,7 +3674,7 @@
         <f>IF(B7=0,0,COUNTIFS('Trade Log'!R:R,A7,'Trade Log'!M:M,"&gt;0")/B7*100)</f>
         <v/>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="11">
         <f>SUMIF('Trade Log'!R:R,A7,'Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3714,7 +3693,7 @@
         <f>IF(B8=0,0,COUNTIFS('Trade Log'!R:R,A8,'Trade Log'!M:M,"&gt;0")/B8*100)</f>
         <v/>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="11">
         <f>SUMIF('Trade Log'!R:R,A8,'Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3733,7 +3712,7 @@
         <f>IF(B9=0,0,COUNTIFS('Trade Log'!R:R,A9,'Trade Log'!M:M,"&gt;0")/B9*100)</f>
         <v/>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="11">
         <f>SUMIF('Trade Log'!R:R,A9,'Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3752,7 +3731,7 @@
         <f>IF(B10=0,0,COUNTIFS('Trade Log'!R:R,A10,'Trade Log'!M:M,"&gt;0")/B10*100)</f>
         <v/>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="11">
         <f>SUMIF('Trade Log'!R:R,A10,'Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3771,7 +3750,7 @@
         <f>IF(B11=0,0,COUNTIFS('Trade Log'!R:R,A11,'Trade Log'!M:M,"&gt;0")/B11*100)</f>
         <v/>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="11">
         <f>SUMIF('Trade Log'!R:R,A11,'Trade Log'!Q:Q)</f>
         <v/>
       </c>
@@ -3801,7 +3780,7 @@
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t>Avg P&amp;L ($)</t>
+          <t>Avg P&amp;L (R)</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3909,6 @@
           <t>60%</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3958,7 +3936,6 @@
           <t>65%</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3986,7 +3963,6 @@
           <t>55%</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>